<commit_message>
Add LinkedIn company URLs to IB banks reference sheet
Resolves each of the 30 banks to its LinkedIn /company/ page (parent entity
for universal banks, where IB employees self-tag) so the IB scraping pipeline
can target them. Slugs for Barclays, BofA, Stifel, and Harris Williams are
best-effort pending a resolve-check.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research/ib-banks-and-offices.xlsx
+++ b/research/ib-banks-and-offices.xlsx
@@ -619,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -661,6 +661,11 @@
           <t># US IB Offices</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>LinkedIn URL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -691,6 +696,11 @@
       <c r="F2" s="6" t="n">
         <v>8</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/goldman-sachs</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -721,6 +731,11 @@
       <c r="F3" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/morgan-stanley</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -751,6 +766,11 @@
       <c r="F4" s="6" t="n">
         <v>7</v>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/jpmorgan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -781,6 +801,11 @@
       <c r="F5" s="6" t="n">
         <v>8</v>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/bank-of-america</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -811,6 +836,11 @@
       <c r="F6" s="6" t="n">
         <v>5</v>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/citi</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -841,6 +871,11 @@
       <c r="F7" s="6" t="n">
         <v>7</v>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/barclays-corporate-and-investment-bank</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -871,6 +906,11 @@
       <c r="F8" s="6" t="n">
         <v>5</v>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/ubs</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -901,6 +941,11 @@
       <c r="F9" s="6" t="n">
         <v>4</v>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/deutsche-bank</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -931,6 +976,11 @@
       <c r="F10" s="6" t="n">
         <v>7</v>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/wells-fargo</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -961,6 +1011,11 @@
       <c r="F11" s="6" t="n">
         <v>11</v>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/rbc-capital-markets</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -991,6 +1046,11 @@
       <c r="F12" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/centerview-partners</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1021,6 +1081,11 @@
       <c r="F13" s="6" t="n">
         <v>10</v>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/evercore</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1051,6 +1116,11 @@
       <c r="F14" s="6" t="n">
         <v>9</v>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/lazard</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1081,6 +1151,11 @@
       <c r="F15" s="6" t="n">
         <v>8</v>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/moelis-&amp;-company</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1111,6 +1186,11 @@
       <c r="F16" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/pjt-partners</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1141,6 +1221,11 @@
       <c r="F17" s="6" t="n">
         <v>8</v>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/perella-weinberg-partners</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1171,6 +1256,11 @@
       <c r="F18" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/qatalyst-partners</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1201,6 +1291,11 @@
       <c r="F19" s="6" t="n">
         <v>7</v>
       </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/guggenheim-securities</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1231,6 +1326,11 @@
       <c r="F20" s="6" t="n">
         <v>4</v>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/rothschild-&amp;-co</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1261,6 +1361,11 @@
       <c r="F21" s="6" t="n">
         <v>13</v>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/jefferies</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1291,6 +1396,11 @@
       <c r="F22" s="6" t="n">
         <v>13</v>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/houlihan-lokey</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1321,6 +1431,11 @@
       <c r="F23" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/william-blair</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1351,6 +1466,11 @@
       <c r="F24" s="6" t="n">
         <v>8</v>
       </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/robert-w-baird-co</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1381,6 +1501,11 @@
       <c r="F25" s="6" t="n">
         <v>9</v>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/harris-williams</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1411,6 +1536,11 @@
       <c r="F26" s="6" t="n">
         <v>10</v>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/piper-sandler</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1441,6 +1571,11 @@
       <c r="F27" s="6" t="n">
         <v>13</v>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/stifel</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1471,6 +1606,11 @@
       <c r="F28" s="6" t="n">
         <v>9</v>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/kbw</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1501,6 +1641,11 @@
       <c r="F29" s="6" t="n">
         <v>7</v>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/raymond-james</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1531,6 +1676,11 @@
       <c r="F30" s="6" t="n">
         <v>11</v>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/lincoln-international</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1560,6 +1710,11 @@
       </c>
       <c r="F31" s="6" t="n">
         <v>5</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/td-cowen</t>
+        </is>
       </c>
     </row>
     <row r="32">

</xml_diff>